<commit_message>
Grava o resultado dos totais e os dados dos gráficos no Excel
O openpyxl salva as fórmulas sem o resultado e os gráficos sem cópia
dos dados; visualizadores que não calculam (celular, prévias online)
mostravam totais e gráficos em branco. Os totais passam a ser calculados
em Python e gravados junto da fórmula, e cada gráfico leva seus dados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SNGhJTcjeFguq5sm6ngrpK
</commit_message>
<xml_diff>
--- a/public/relatorio.xlsx
+++ b/public/relatorio.xlsx
@@ -376,6 +376,12 @@
           <tx>
             <strRef>
               <f>'Resumo'!B14</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Faturamento líquido</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -387,13 +393,38 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumo'!$A$15:$A$17</f>
-            </numRef>
+              <strCache>
+                <ptCount val="3"/>
+                <pt idx="0">
+                  <v>Centro</v>
+                </pt>
+                <pt idx="1">
+                  <v>Umarizal</v>
+                </pt>
+                <pt idx="2">
+                  <v>Ananindeua</v>
+                </pt>
+              </strCache>
+            </strRef>
           </cat>
           <val>
             <numRef>
               <f>'Resumo'!$B$15:$B$17</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00;[Red]-"R$" #,##0.00</formatCode>
+                <ptCount val="3"/>
+                <pt idx="0">
+                  <v>43538.89</v>
+                </pt>
+                <pt idx="1">
+                  <v>32849.73</v>
+                </pt>
+                <pt idx="2">
+                  <v>27462.95</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -403,6 +434,12 @@
           <tx>
             <strRef>
               <f>'Resumo'!C14</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Meta</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -414,13 +451,38 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumo'!$A$15:$A$17</f>
-            </numRef>
+              <strCache>
+                <ptCount val="3"/>
+                <pt idx="0">
+                  <v>Centro</v>
+                </pt>
+                <pt idx="1">
+                  <v>Umarizal</v>
+                </pt>
+                <pt idx="2">
+                  <v>Ananindeua</v>
+                </pt>
+              </strCache>
+            </strRef>
           </cat>
           <val>
             <numRef>
               <f>'Resumo'!$C$15:$C$17</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00;[Red]-"R$" #,##0.00</formatCode>
+                <ptCount val="3"/>
+                <pt idx="0">
+                  <v>47000</v>
+                </pt>
+                <pt idx="1">
+                  <v>40000</v>
+                </pt>
+                <pt idx="2">
+                  <v>27000</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -491,6 +553,12 @@
           <tx>
             <strRef>
               <f>'Resumo'!B21</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Faturamento líquido</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -502,13 +570,50 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumo'!$A$22:$A$26</f>
-            </numRef>
+              <strCache>
+                <ptCount val="5"/>
+                <pt idx="0">
+                  <v>Dermatológicos</v>
+                </pt>
+                <pt idx="1">
+                  <v>Cápsulas e suplementos</v>
+                </pt>
+                <pt idx="2">
+                  <v>Veterinários</v>
+                </pt>
+                <pt idx="3">
+                  <v>Florais e homeopatia</v>
+                </pt>
+                <pt idx="4">
+                  <v>Revenda</v>
+                </pt>
+              </strCache>
+            </strRef>
           </cat>
           <val>
             <numRef>
               <f>'Resumo'!$B$22:$B$26</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00;[Red]-"R$" #,##0.00</formatCode>
+                <ptCount val="5"/>
+                <pt idx="0">
+                  <v>44268.49</v>
+                </pt>
+                <pt idx="1">
+                  <v>36645.1</v>
+                </pt>
+                <pt idx="2">
+                  <v>8699.5</v>
+                </pt>
+                <pt idx="3">
+                  <v>7150.06</v>
+                </pt>
+                <pt idx="4">
+                  <v>7088.42</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -576,6 +681,12 @@
           <tx>
             <strRef>
               <f>'Vendas por dia'!C4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Centro</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -589,11 +700,175 @@
           <cat>
             <numRef>
               <f>'Vendas por dia'!$A$5:$A$30</f>
+              <numCache>
+                <formatCode>dd/mm/yyyy</formatCode>
+                <ptCount val="26"/>
+                <pt idx="0">
+                  <v>46235</v>
+                </pt>
+                <pt idx="1">
+                  <v>46237</v>
+                </pt>
+                <pt idx="2">
+                  <v>46238</v>
+                </pt>
+                <pt idx="3">
+                  <v>46239</v>
+                </pt>
+                <pt idx="4">
+                  <v>46240</v>
+                </pt>
+                <pt idx="5">
+                  <v>46241</v>
+                </pt>
+                <pt idx="6">
+                  <v>46242</v>
+                </pt>
+                <pt idx="7">
+                  <v>46244</v>
+                </pt>
+                <pt idx="8">
+                  <v>46245</v>
+                </pt>
+                <pt idx="9">
+                  <v>46246</v>
+                </pt>
+                <pt idx="10">
+                  <v>46247</v>
+                </pt>
+                <pt idx="11">
+                  <v>46248</v>
+                </pt>
+                <pt idx="12">
+                  <v>46249</v>
+                </pt>
+                <pt idx="13">
+                  <v>46251</v>
+                </pt>
+                <pt idx="14">
+                  <v>46252</v>
+                </pt>
+                <pt idx="15">
+                  <v>46253</v>
+                </pt>
+                <pt idx="16">
+                  <v>46254</v>
+                </pt>
+                <pt idx="17">
+                  <v>46255</v>
+                </pt>
+                <pt idx="18">
+                  <v>46256</v>
+                </pt>
+                <pt idx="19">
+                  <v>46258</v>
+                </pt>
+                <pt idx="20">
+                  <v>46259</v>
+                </pt>
+                <pt idx="21">
+                  <v>46260</v>
+                </pt>
+                <pt idx="22">
+                  <v>46261</v>
+                </pt>
+                <pt idx="23">
+                  <v>46262</v>
+                </pt>
+                <pt idx="24">
+                  <v>46263</v>
+                </pt>
+                <pt idx="25">
+                  <v>46265</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Vendas por dia'!$C$5:$C$30</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00;[Red]-"R$" #,##0.00</formatCode>
+                <ptCount val="26"/>
+                <pt idx="0">
+                  <v>988.85</v>
+                </pt>
+                <pt idx="1">
+                  <v>2612.72</v>
+                </pt>
+                <pt idx="2">
+                  <v>1167.61</v>
+                </pt>
+                <pt idx="3">
+                  <v>1905.21</v>
+                </pt>
+                <pt idx="4">
+                  <v>1465.62</v>
+                </pt>
+                <pt idx="5">
+                  <v>1428.9</v>
+                </pt>
+                <pt idx="6">
+                  <v>1473.57</v>
+                </pt>
+                <pt idx="7">
+                  <v>2052</v>
+                </pt>
+                <pt idx="8">
+                  <v>2205.69</v>
+                </pt>
+                <pt idx="9">
+                  <v>1982.39</v>
+                </pt>
+                <pt idx="10">
+                  <v>1453.94</v>
+                </pt>
+                <pt idx="11">
+                  <v>1713.36</v>
+                </pt>
+                <pt idx="12">
+                  <v>1130.46</v>
+                </pt>
+                <pt idx="13">
+                  <v>1552.25</v>
+                </pt>
+                <pt idx="14">
+                  <v>1472.13</v>
+                </pt>
+                <pt idx="15">
+                  <v>2285.54</v>
+                </pt>
+                <pt idx="16">
+                  <v>2291.28</v>
+                </pt>
+                <pt idx="17">
+                  <v>1471.7</v>
+                </pt>
+                <pt idx="18">
+                  <v>899.74</v>
+                </pt>
+                <pt idx="19">
+                  <v>1697.36</v>
+                </pt>
+                <pt idx="20">
+                  <v>1584.94</v>
+                </pt>
+                <pt idx="21">
+                  <v>1666.35</v>
+                </pt>
+                <pt idx="22">
+                  <v>2683.68</v>
+                </pt>
+                <pt idx="23">
+                  <v>1710.31</v>
+                </pt>
+                <pt idx="24">
+                  <v>925.88</v>
+                </pt>
+                <pt idx="25">
+                  <v>1717.41</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -603,6 +878,12 @@
           <tx>
             <strRef>
               <f>'Vendas por dia'!D4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Umarizal</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -616,11 +897,175 @@
           <cat>
             <numRef>
               <f>'Vendas por dia'!$A$5:$A$30</f>
+              <numCache>
+                <formatCode>dd/mm/yyyy</formatCode>
+                <ptCount val="26"/>
+                <pt idx="0">
+                  <v>46235</v>
+                </pt>
+                <pt idx="1">
+                  <v>46237</v>
+                </pt>
+                <pt idx="2">
+                  <v>46238</v>
+                </pt>
+                <pt idx="3">
+                  <v>46239</v>
+                </pt>
+                <pt idx="4">
+                  <v>46240</v>
+                </pt>
+                <pt idx="5">
+                  <v>46241</v>
+                </pt>
+                <pt idx="6">
+                  <v>46242</v>
+                </pt>
+                <pt idx="7">
+                  <v>46244</v>
+                </pt>
+                <pt idx="8">
+                  <v>46245</v>
+                </pt>
+                <pt idx="9">
+                  <v>46246</v>
+                </pt>
+                <pt idx="10">
+                  <v>46247</v>
+                </pt>
+                <pt idx="11">
+                  <v>46248</v>
+                </pt>
+                <pt idx="12">
+                  <v>46249</v>
+                </pt>
+                <pt idx="13">
+                  <v>46251</v>
+                </pt>
+                <pt idx="14">
+                  <v>46252</v>
+                </pt>
+                <pt idx="15">
+                  <v>46253</v>
+                </pt>
+                <pt idx="16">
+                  <v>46254</v>
+                </pt>
+                <pt idx="17">
+                  <v>46255</v>
+                </pt>
+                <pt idx="18">
+                  <v>46256</v>
+                </pt>
+                <pt idx="19">
+                  <v>46258</v>
+                </pt>
+                <pt idx="20">
+                  <v>46259</v>
+                </pt>
+                <pt idx="21">
+                  <v>46260</v>
+                </pt>
+                <pt idx="22">
+                  <v>46261</v>
+                </pt>
+                <pt idx="23">
+                  <v>46262</v>
+                </pt>
+                <pt idx="24">
+                  <v>46263</v>
+                </pt>
+                <pt idx="25">
+                  <v>46265</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Vendas por dia'!$D$5:$D$30</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00;[Red]-"R$" #,##0.00</formatCode>
+                <ptCount val="26"/>
+                <pt idx="0">
+                  <v>559.4</v>
+                </pt>
+                <pt idx="1">
+                  <v>1457.29</v>
+                </pt>
+                <pt idx="2">
+                  <v>929.85</v>
+                </pt>
+                <pt idx="3">
+                  <v>1480.09</v>
+                </pt>
+                <pt idx="4">
+                  <v>1871.21</v>
+                </pt>
+                <pt idx="5">
+                  <v>1037.95</v>
+                </pt>
+                <pt idx="6">
+                  <v>883.6799999999999</v>
+                </pt>
+                <pt idx="7">
+                  <v>1154.87</v>
+                </pt>
+                <pt idx="8">
+                  <v>1786.41</v>
+                </pt>
+                <pt idx="9">
+                  <v>1222.95</v>
+                </pt>
+                <pt idx="10">
+                  <v>1237.51</v>
+                </pt>
+                <pt idx="11">
+                  <v>1213.85</v>
+                </pt>
+                <pt idx="12">
+                  <v>791.7</v>
+                </pt>
+                <pt idx="13">
+                  <v>1514.23</v>
+                </pt>
+                <pt idx="14">
+                  <v>2468.68</v>
+                </pt>
+                <pt idx="15">
+                  <v>1622.2</v>
+                </pt>
+                <pt idx="16">
+                  <v>1155.63</v>
+                </pt>
+                <pt idx="17">
+                  <v>1142.79</v>
+                </pt>
+                <pt idx="18">
+                  <v>1371.08</v>
+                </pt>
+                <pt idx="19">
+                  <v>1665.05</v>
+                </pt>
+                <pt idx="20">
+                  <v>987.04</v>
+                </pt>
+                <pt idx="21">
+                  <v>1309.55</v>
+                </pt>
+                <pt idx="22">
+                  <v>1451.54</v>
+                </pt>
+                <pt idx="23">
+                  <v>826.76</v>
+                </pt>
+                <pt idx="24">
+                  <v>722.42</v>
+                </pt>
+                <pt idx="25">
+                  <v>986</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -630,6 +1075,12 @@
           <tx>
             <strRef>
               <f>'Vendas por dia'!E4</f>
+              <strCache>
+                <ptCount val="1"/>
+                <pt idx="0">
+                  <v>Ananindeua</v>
+                </pt>
+              </strCache>
             </strRef>
           </tx>
           <spPr>
@@ -643,11 +1094,175 @@
           <cat>
             <numRef>
               <f>'Vendas por dia'!$A$5:$A$30</f>
+              <numCache>
+                <formatCode>dd/mm/yyyy</formatCode>
+                <ptCount val="26"/>
+                <pt idx="0">
+                  <v>46235</v>
+                </pt>
+                <pt idx="1">
+                  <v>46237</v>
+                </pt>
+                <pt idx="2">
+                  <v>46238</v>
+                </pt>
+                <pt idx="3">
+                  <v>46239</v>
+                </pt>
+                <pt idx="4">
+                  <v>46240</v>
+                </pt>
+                <pt idx="5">
+                  <v>46241</v>
+                </pt>
+                <pt idx="6">
+                  <v>46242</v>
+                </pt>
+                <pt idx="7">
+                  <v>46244</v>
+                </pt>
+                <pt idx="8">
+                  <v>46245</v>
+                </pt>
+                <pt idx="9">
+                  <v>46246</v>
+                </pt>
+                <pt idx="10">
+                  <v>46247</v>
+                </pt>
+                <pt idx="11">
+                  <v>46248</v>
+                </pt>
+                <pt idx="12">
+                  <v>46249</v>
+                </pt>
+                <pt idx="13">
+                  <v>46251</v>
+                </pt>
+                <pt idx="14">
+                  <v>46252</v>
+                </pt>
+                <pt idx="15">
+                  <v>46253</v>
+                </pt>
+                <pt idx="16">
+                  <v>46254</v>
+                </pt>
+                <pt idx="17">
+                  <v>46255</v>
+                </pt>
+                <pt idx="18">
+                  <v>46256</v>
+                </pt>
+                <pt idx="19">
+                  <v>46258</v>
+                </pt>
+                <pt idx="20">
+                  <v>46259</v>
+                </pt>
+                <pt idx="21">
+                  <v>46260</v>
+                </pt>
+                <pt idx="22">
+                  <v>46261</v>
+                </pt>
+                <pt idx="23">
+                  <v>46262</v>
+                </pt>
+                <pt idx="24">
+                  <v>46263</v>
+                </pt>
+                <pt idx="25">
+                  <v>46265</v>
+                </pt>
+              </numCache>
             </numRef>
           </cat>
           <val>
             <numRef>
               <f>'Vendas por dia'!$E$5:$E$30</f>
+              <numCache>
+                <formatCode>"R$" #,##0.00;[Red]-"R$" #,##0.00</formatCode>
+                <ptCount val="26"/>
+                <pt idx="0">
+                  <v>570.71</v>
+                </pt>
+                <pt idx="1">
+                  <v>1589.46</v>
+                </pt>
+                <pt idx="2">
+                  <v>675.28</v>
+                </pt>
+                <pt idx="3">
+                  <v>1589.93</v>
+                </pt>
+                <pt idx="4">
+                  <v>987.53</v>
+                </pt>
+                <pt idx="5">
+                  <v>1343.87</v>
+                </pt>
+                <pt idx="6">
+                  <v>720.38</v>
+                </pt>
+                <pt idx="7">
+                  <v>1343.53</v>
+                </pt>
+                <pt idx="8">
+                  <v>1091.17</v>
+                </pt>
+                <pt idx="9">
+                  <v>933.36</v>
+                </pt>
+                <pt idx="10">
+                  <v>1020.63</v>
+                </pt>
+                <pt idx="11">
+                  <v>943.8</v>
+                </pt>
+                <pt idx="12">
+                  <v>476.53</v>
+                </pt>
+                <pt idx="13">
+                  <v>1079.46</v>
+                </pt>
+                <pt idx="14">
+                  <v>1289.15</v>
+                </pt>
+                <pt idx="15">
+                  <v>1067.61</v>
+                </pt>
+                <pt idx="16">
+                  <v>898.14</v>
+                </pt>
+                <pt idx="17">
+                  <v>1185.96</v>
+                </pt>
+                <pt idx="18">
+                  <v>345.86</v>
+                </pt>
+                <pt idx="19">
+                  <v>1341.92</v>
+                </pt>
+                <pt idx="20">
+                  <v>1144.3</v>
+                </pt>
+                <pt idx="21">
+                  <v>1004.55</v>
+                </pt>
+                <pt idx="22">
+                  <v>1739.2</v>
+                </pt>
+                <pt idx="23">
+                  <v>1289.61</v>
+                </pt>
+                <pt idx="24">
+                  <v>418.54</v>
+                </pt>
+                <pt idx="25">
+                  <v>1372.47</v>
+                </pt>
+              </numCache>
             </numRef>
           </val>
         </ser>
@@ -1726,7 +2341,7 @@
       </c>
       <c r="F5" s="30">
         <f>SUM(C5:E5)</f>
-        <v/>
+        <v>2118.96</v>
       </c>
     </row>
     <row r="6">
@@ -1749,7 +2364,7 @@
       </c>
       <c r="F6" s="32">
         <f>SUM(C6:E6)</f>
-        <v/>
+        <v>5659.47</v>
       </c>
     </row>
     <row r="7">
@@ -1772,7 +2387,7 @@
       </c>
       <c r="F7" s="30">
         <f>SUM(C7:E7)</f>
-        <v/>
+        <v>2772.74</v>
       </c>
     </row>
     <row r="8">
@@ -1795,7 +2410,7 @@
       </c>
       <c r="F8" s="32">
         <f>SUM(C8:E8)</f>
-        <v/>
+        <v>4975.23</v>
       </c>
     </row>
     <row r="9">
@@ -1818,7 +2433,7 @@
       </c>
       <c r="F9" s="30">
         <f>SUM(C9:E9)</f>
-        <v/>
+        <v>4324.36</v>
       </c>
     </row>
     <row r="10">
@@ -1841,7 +2456,7 @@
       </c>
       <c r="F10" s="32">
         <f>SUM(C10:E10)</f>
-        <v/>
+        <v>3810.72</v>
       </c>
     </row>
     <row r="11">
@@ -1864,7 +2479,7 @@
       </c>
       <c r="F11" s="30">
         <f>SUM(C11:E11)</f>
-        <v/>
+        <v>3077.63</v>
       </c>
     </row>
     <row r="12">
@@ -1887,7 +2502,7 @@
       </c>
       <c r="F12" s="32">
         <f>SUM(C12:E12)</f>
-        <v/>
+        <v>4550.4</v>
       </c>
     </row>
     <row r="13">
@@ -1910,7 +2525,7 @@
       </c>
       <c r="F13" s="30">
         <f>SUM(C13:E13)</f>
-        <v/>
+        <v>5083.27</v>
       </c>
     </row>
     <row r="14">
@@ -1933,7 +2548,7 @@
       </c>
       <c r="F14" s="32">
         <f>SUM(C14:E14)</f>
-        <v/>
+        <v>4138.7</v>
       </c>
     </row>
     <row r="15">
@@ -1956,7 +2571,7 @@
       </c>
       <c r="F15" s="30">
         <f>SUM(C15:E15)</f>
-        <v/>
+        <v>3712.08</v>
       </c>
     </row>
     <row r="16">
@@ -1979,7 +2594,7 @@
       </c>
       <c r="F16" s="32">
         <f>SUM(C16:E16)</f>
-        <v/>
+        <v>3871.01</v>
       </c>
     </row>
     <row r="17">
@@ -2002,7 +2617,7 @@
       </c>
       <c r="F17" s="30">
         <f>SUM(C17:E17)</f>
-        <v/>
+        <v>2398.69</v>
       </c>
     </row>
     <row r="18">
@@ -2025,7 +2640,7 @@
       </c>
       <c r="F18" s="32">
         <f>SUM(C18:E18)</f>
-        <v/>
+        <v>4145.94</v>
       </c>
     </row>
     <row r="19">
@@ -2048,7 +2663,7 @@
       </c>
       <c r="F19" s="30">
         <f>SUM(C19:E19)</f>
-        <v/>
+        <v>5229.96</v>
       </c>
     </row>
     <row r="20">
@@ -2071,7 +2686,7 @@
       </c>
       <c r="F20" s="32">
         <f>SUM(C20:E20)</f>
-        <v/>
+        <v>4975.35</v>
       </c>
     </row>
     <row r="21">
@@ -2094,7 +2709,7 @@
       </c>
       <c r="F21" s="30">
         <f>SUM(C21:E21)</f>
-        <v/>
+        <v>4345.05</v>
       </c>
     </row>
     <row r="22">
@@ -2117,7 +2732,7 @@
       </c>
       <c r="F22" s="32">
         <f>SUM(C22:E22)</f>
-        <v/>
+        <v>3800.45</v>
       </c>
     </row>
     <row r="23">
@@ -2140,7 +2755,7 @@
       </c>
       <c r="F23" s="30">
         <f>SUM(C23:E23)</f>
-        <v/>
+        <v>2616.68</v>
       </c>
     </row>
     <row r="24">
@@ -2163,7 +2778,7 @@
       </c>
       <c r="F24" s="32">
         <f>SUM(C24:E24)</f>
-        <v/>
+        <v>4704.33</v>
       </c>
     </row>
     <row r="25">
@@ -2186,7 +2801,7 @@
       </c>
       <c r="F25" s="30">
         <f>SUM(C25:E25)</f>
-        <v/>
+        <v>3716.28</v>
       </c>
     </row>
     <row r="26">
@@ -2209,7 +2824,7 @@
       </c>
       <c r="F26" s="32">
         <f>SUM(C26:E26)</f>
-        <v/>
+        <v>3980.45</v>
       </c>
     </row>
     <row r="27">
@@ -2232,7 +2847,7 @@
       </c>
       <c r="F27" s="30">
         <f>SUM(C27:E27)</f>
-        <v/>
+        <v>5874.42</v>
       </c>
     </row>
     <row r="28">
@@ -2255,7 +2870,7 @@
       </c>
       <c r="F28" s="32">
         <f>SUM(C28:E28)</f>
-        <v/>
+        <v>3826.68</v>
       </c>
     </row>
     <row r="29">
@@ -2278,7 +2893,7 @@
       </c>
       <c r="F29" s="30">
         <f>SUM(C29:E29)</f>
-        <v/>
+        <v>2066.84</v>
       </c>
     </row>
     <row r="30">
@@ -2301,7 +2916,7 @@
       </c>
       <c r="F30" s="32">
         <f>SUM(C30:E30)</f>
-        <v/>
+        <v>4075.88</v>
       </c>
     </row>
     <row r="31">
@@ -2313,19 +2928,19 @@
       <c r="B31" s="22" t="n"/>
       <c r="C31" s="23">
         <f>SUM(C5:C30)</f>
-        <v/>
+        <v>43538.89</v>
       </c>
       <c r="D31" s="23">
         <f>SUM(D5:D30)</f>
-        <v/>
+        <v>32849.73</v>
       </c>
       <c r="E31" s="23">
         <f>SUM(E5:E30)</f>
-        <v/>
+        <v>27462.95</v>
       </c>
       <c r="F31" s="23">
         <f>SUM(F5:F30)</f>
-        <v/>
+        <v>103851.57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>